<commit_message>
perf(import): optimasi memory dan query pada proses import excel
- Membersihkan kolom hantu 16.384 (XFD) pada file template excel (guru, kelas, mapel)
- Menambahkan auto-sanitize file upload untuk memotong kolom hantu sebelum dibaca PhpSpreadsheet
</commit_message>
<xml_diff>
--- a/public/templates/template_guru.xlsx
+++ b/public/templates/template_guru.xlsx
@@ -418,12 +418,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -433,11 +432,6 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>